<commit_message>
fix: scanAffairsBatchRow 时间字段用 time.Time
</commit_message>
<xml_diff>
--- a/docs/alliance-templates/alliance-achievements.xlsx
+++ b/docs/alliance-templates/alliance-achievements.xlsx
@@ -1,98 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="true" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合作成果" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'Sheet1'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合作成果'!$A$2:$D$2</definedName>
   </definedNames>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="122211" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>成果名称</t>
-  </si>
-  <si>
-    <t>成果类型</t>
-  </si>
-  <si>
-    <t>描述</t>
-  </si>
-  <si>
-    <t>成果日期</t>
-  </si>
-  <si>
-    <t>AI算法工程师岗位标准</t>
-  </si>
-  <si>
-    <t>job</t>
-  </si>
-  <si>
-    <t>联合制定AI算法工程师岗位能力标准与培养方案</t>
-  </si>
-  <si>
-    <t>2026-05-20</t>
-  </si>
-  <si>
-    <t>智慧工厂实践场景</t>
-  </si>
-  <si>
-    <t>scene</t>
-  </si>
-  <si>
-    <t>建成智慧工厂数字孪生实践场景，覆盖5个典型工序</t>
-  </si>
-  <si>
-    <t>2026-03-15</t>
-  </si>
-  <si>
-    <t>Python数据分析课程包</t>
-  </si>
-  <si>
-    <t>course</t>
-  </si>
-  <si>
-    <t>校企联合开发Python数据分析课程15学时，含配套实训项目</t>
-  </si>
-  <si>
-    <t>2026-04-10</t>
-  </si>
-  <si>
-    <t>产教融合案例集</t>
-  </si>
-  <si>
-    <t>custom</t>
-  </si>
-  <si>
-    <t>收录校企合作优秀案例20篇，出版产教融合案例集</t>
-  </si>
-  <si>
-    <t>2026-06-01</t>
-  </si>
-  <si>
-    <t>5G通信实训平台</t>
-  </si>
-  <si>
-    <t>建成5G通信网络部署与优化实训平台</t>
-  </si>
-  <si>
-    <t>2026-02-28</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -102,13 +28,23 @@
     <font>
       <family val="2"/>
       <b val="1"/>
-      <color/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -118,8 +54,20 @@
         <fgColor rgb="FFCCE5FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -128,24 +76,113 @@
       <diagonal/>
     </border>
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="false">
-      <alignment/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -406,102 +443,171 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr filterMode="true"/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="30"/>
-    <col customWidth="true" max="2" min="2" width="14"/>
-    <col customWidth="true" max="3" min="3" width="50"/>
-    <col customWidth="true" max="4" min="4" width="14"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="true">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
+    <row r="1" ht="112" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>填写说明：
+* 必填列。
+成果类型：job（岗位） / scene（场景） / course（课程） / custom（自定义），默认为 custom
+描述：文本，选填
+成果日期：格式 YYYY-MM-DD，选填</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
     </row>
-    <row r="2" ht="20" customHeight="true">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>成果名称 *</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>成果类型</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>成果日期</t>
+        </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="true">
-      <c r="A3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>11</v>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>AI算法工程师岗位标准</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>job</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>联合制定AI算法工程师岗位能力标准与培养方案</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="true">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>15</v>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>智慧工厂实践场景</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>scene</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>建成智慧工厂数字孪生实践场景，覆盖5个典型工序</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="true">
-      <c r="A5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>19</v>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Python数据分析课程包</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>course</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>校企联合开发Python数据分析课程15学时，含配套实训项目</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="true">
-      <c r="A6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>22</v>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>产教融合案例集</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>收录校企合作优秀案例20篇，出版产教融合案例集</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>5G通信实训平台</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>scene</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>建成5G通信网络部署与优化实训平台</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$D$6"/>
+  <autoFilter ref="A2:D2"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>